<commit_message>
After making separate copy of Poland Hire for PK14 and PK17
</commit_message>
<xml_diff>
--- a/Data/Hires/Workday_NewHire_Portugal_Regression_PK14.xlsx
+++ b/Data/Hires/Workday_NewHire_Portugal_Regression_PK14.xlsx
@@ -1,23 +1,38 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27928"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{644F0A33-05B5-4B06-A8B0-006B060720A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1068" yWindow="-108" windowWidth="22080" windowHeight="13176"/>
+    <workbookView xWindow="1068" yWindow="-108" windowWidth="22080" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Sheet1" state="visible" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase">Sheet1!$A$1:$BY$53</definedName>
   </definedNames>
-  <calcPr calcId="171027"/>
+  <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="881" uniqueCount="200">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="907" uniqueCount="215">
   <si>
     <t>TestCaseIDs</t>
   </si>
@@ -214,7 +229,7 @@
     <t>Test_1</t>
   </si>
   <si>
-    <t>10697805</t>
+    <t>10697810</t>
   </si>
   <si>
     <t>Passed</t>
@@ -229,210 +244,220 @@
     <t>PortugalOne</t>
   </si>
   <si>
+    <t>DryRunThirdB</t>
+  </si>
+  <si>
+    <t>Sr.</t>
+  </si>
+  <si>
+    <t>Landline</t>
+  </si>
+  <si>
+    <t>Home</t>
+  </si>
+  <si>
+    <t>Automation Street Name</t>
+  </si>
+  <si>
+    <t>4000-087</t>
+  </si>
+  <si>
+    <t>Porto</t>
+  </si>
+  <si>
+    <t>Street Address</t>
+  </si>
+  <si>
+    <t>automation@qe.com</t>
+  </si>
+  <si>
+    <t>New Hire</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Permanent</t>
+  </si>
+  <si>
+    <t>Retail Assistant</t>
+  </si>
+  <si>
+    <t>Full Time</t>
+  </si>
+  <si>
+    <t>420 Lisbon - UBBO</t>
+  </si>
+  <si>
+    <t>1.A.1 - Cto 6 Meses- Abertura Loja- RA/SUP-FT (Contratos RA &amp; Supervisores Portugal-Portugal) (Contratos RA &amp; Supervisores Portugal-Portugal)@401</t>
+  </si>
+  <si>
+    <t>5 Dias</t>
+  </si>
+  <si>
+    <t>N/A</t>
+  </si>
+  <si>
+    <t>94 Retail Operatives</t>
+  </si>
+  <si>
+    <t>01 Accessories</t>
+  </si>
+  <si>
+    <t>PT Monthly</t>
+  </si>
+  <si>
+    <t>Pensões-Casado-Dois Tit.-Deficiente</t>
+  </si>
+  <si>
+    <t>312-ENSINO SECUNDARIO TECNICO COMPLEMENTAR</t>
+  </si>
+  <si>
+    <t>Acréscimo excepcional de actividade da empresa</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>Sem Termo (FT) - Permanente</t>
+  </si>
+  <si>
+    <t>Defaulted</t>
+  </si>
+  <si>
+    <t>Portugal Retail Assistant</t>
+  </si>
+  <si>
+    <t>Operador de supermercado de 1</t>
+  </si>
+  <si>
+    <t>Male</t>
+  </si>
+  <si>
+    <t>01/01/1999</t>
+  </si>
+  <si>
+    <t>Guarda</t>
+  </si>
+  <si>
+    <t>Married</t>
+  </si>
+  <si>
+    <t>26/01/2019</t>
+  </si>
+  <si>
+    <t>Social Security Identification Number (NISS)</t>
+  </si>
+  <si>
+    <t>Taxpayer ID Number (NIF)</t>
+  </si>
+  <si>
+    <t>ID Number (Numero de</t>
+  </si>
+  <si>
+    <t>24982928 2AP28</t>
+  </si>
+  <si>
+    <t>BBVAESMM128</t>
+  </si>
+  <si>
+    <t>Checking</t>
+  </si>
+  <si>
+    <t>PT50000201231234567890154</t>
+  </si>
+  <si>
+    <t>Test_2</t>
+  </si>
+  <si>
+    <t>10697812</t>
+  </si>
+  <si>
+    <t>420 Store Management (Veved Jepela (4206015))</t>
+  </si>
+  <si>
+    <t>PortugalTwo</t>
+  </si>
+  <si>
+    <t>DryRunThirdA</t>
+  </si>
+  <si>
+    <t>Sra.</t>
+  </si>
+  <si>
+    <t>New</t>
+  </si>
+  <si>
+    <t>Auto 80659064</t>
+  </si>
+  <si>
+    <t>Store Manager</t>
+  </si>
+  <si>
+    <t>92 Retail Management</t>
+  </si>
+  <si>
+    <t>Actividade sazonal ou outra cujo ciclo anual de produção apresente irregularidades decorrentes da natureza estrutural do respectivo mercado, incluindo o abastecimento de matéria-prima</t>
+  </si>
+  <si>
+    <t>Female</t>
+  </si>
+  <si>
+    <t>Single</t>
+  </si>
+  <si>
+    <t>24982928 2AP27</t>
+  </si>
+  <si>
+    <t>Test_3</t>
+  </si>
+  <si>
+    <t>10697813</t>
+  </si>
+  <si>
+    <t>PortugalThree</t>
+  </si>
+  <si>
     <t>DryRunThird</t>
   </si>
   <si>
-    <t>Sr.</t>
-  </si>
-  <si>
-    <t>Landline</t>
-  </si>
-  <si>
-    <t>Home</t>
-  </si>
-  <si>
-    <t>Automation Street Name</t>
-  </si>
-  <si>
-    <t>4000-087</t>
-  </si>
-  <si>
-    <t>Porto</t>
-  </si>
-  <si>
-    <t>Street Address</t>
-  </si>
-  <si>
-    <t>automation@qe.com</t>
-  </si>
-  <si>
-    <t>New Hire</t>
-  </si>
-  <si>
-    <t>No</t>
-  </si>
-  <si>
-    <t>Permanent</t>
-  </si>
-  <si>
-    <t>Retail Assistant</t>
-  </si>
-  <si>
-    <t>Full Time</t>
-  </si>
-  <si>
-    <t>420 Lisbon - UBBO</t>
-  </si>
-  <si>
-    <t>1.A.1 - Cto 6 Meses- Abertura Loja- RA/SUP-FT (Contratos RA &amp; Supervisores Portugal-Portugal) (Contratos RA &amp; Supervisores Portugal-Portugal)@401</t>
-  </si>
-  <si>
-    <t>5 Dias</t>
-  </si>
-  <si>
-    <t>N/A</t>
-  </si>
-  <si>
-    <t>94 Retail Operatives</t>
-  </si>
-  <si>
-    <t>01 Accessories</t>
-  </si>
-  <si>
-    <t>PT Monthly</t>
-  </si>
-  <si>
-    <t>Pensões-Casado-Dois Tit.-Deficiente</t>
-  </si>
-  <si>
-    <t>312-ENSINO SECUNDARIO TECNICO COMPLEMENTAR</t>
-  </si>
-  <si>
-    <t>Acréscimo excepcional de actividade da empresa</t>
-  </si>
-  <si>
-    <t>Active</t>
-  </si>
-  <si>
-    <t>Sem Termo (FT) - Permanente</t>
-  </si>
-  <si>
-    <t>Defaulted</t>
-  </si>
-  <si>
-    <t>Portugal Retail Assistant</t>
-  </si>
-  <si>
-    <t>Operador de supermercado de 1</t>
-  </si>
-  <si>
-    <t>Male</t>
-  </si>
-  <si>
-    <t>01/01/1999</t>
-  </si>
-  <si>
-    <t>Guarda</t>
-  </si>
-  <si>
-    <t>Married</t>
-  </si>
-  <si>
-    <t>26/01/2019</t>
-  </si>
-  <si>
-    <t>Social Security Identification Number (NISS)</t>
-  </si>
-  <si>
-    <t>Taxpayer ID Number (NIF)</t>
-  </si>
-  <si>
-    <t>ID Number (Numero de</t>
-  </si>
-  <si>
-    <t>24982928 2AP11</t>
-  </si>
-  <si>
-    <t>BBVAESMM128</t>
-  </si>
-  <si>
-    <t>Checking</t>
-  </si>
-  <si>
-    <t>PT50000201231234567890154</t>
-  </si>
-  <si>
-    <t>Test_2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Test failed for 'PortugalTwo DryRunThird' Employee:{10697806}Error: locator.isVisible: Error: strict mode violation: locator('text=Success! Event approved') resolved to 2 elements:
-    1) &lt;h2 data-automation-id="" title="Success! Event appr…&gt;Success! Event approved&lt;/h2&gt; aka getByRole('heading', { name: 'Success! Event approved' }).first()
-    2) &lt;h2 data-automation-id="" title="Success! Event appr…&gt;Success! Event approved&lt;/h2&gt; aka getByRole('heading', { name: 'Success! Event approved' }).nth(1)
+    <t>Intern</t>
+  </si>
+  <si>
+    <t>Part Time</t>
+  </si>
+  <si>
+    <t>261 Tills</t>
+  </si>
+  <si>
+    <t>Contratação de trabalhadores à procura de primeiro emprego, em situação de desemprego de longa duração ou noutra prevista em legislação especial de política de emprego (só aplicável para contrato a termo certo)</t>
+  </si>
+  <si>
+    <t>Termo Incerto (PT) - Temporário</t>
+  </si>
+  <si>
+    <t>Operador ajudante do 1</t>
+  </si>
+  <si>
+    <t>24982928 2AP13</t>
+  </si>
+  <si>
+    <t>Test_4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Test failed for 'PortugalFour DryRunThird' Employee:{}TimeoutError: locator.click: Timeout 30000ms exceeded.
 Call log:
-  [2m-   checking visibility of locator('text=Success! Event approved')[22m
+  [2m- waiting for getByLabel('Prefix')[22m
 </t>
   </si>
   <si>
     <t>Failed</t>
   </si>
   <si>
-    <t>420 Store Management (Veved Jepela (4206015))</t>
-  </si>
-  <si>
-    <t>PortugalTwo</t>
-  </si>
-  <si>
-    <t>Sra.</t>
-  </si>
-  <si>
-    <t>New</t>
-  </si>
-  <si>
-    <t>Auto 13403961</t>
-  </si>
-  <si>
-    <t>Store Manager</t>
-  </si>
-  <si>
-    <t>92 Retail Management</t>
-  </si>
-  <si>
-    <t>Actividade sazonal ou outra cujo ciclo anual de produção apresente irregularidades decorrentes da natureza estrutural do respectivo mercado, incluindo o abastecimento de matéria-prima</t>
-  </si>
-  <si>
-    <t>Female</t>
-  </si>
-  <si>
-    <t>Single</t>
-  </si>
-  <si>
-    <t>24982928 2AP12</t>
-  </si>
-  <si>
-    <t>Test_3</t>
-  </si>
-  <si>
-    <t>PortugalThree</t>
-  </si>
-  <si>
-    <t>Intern (Fixed Term)</t>
-  </si>
-  <si>
-    <t>Part Time</t>
-  </si>
-  <si>
-    <t>261 Tills</t>
-  </si>
-  <si>
-    <t>Contratação de trabalhadores à procura de primeiro emprego, em situação de desemprego de longa duração ou noutra prevista em legislação especial de política de emprego (só aplicável para contrato a termo certo)</t>
-  </si>
-  <si>
-    <t>Termo Incerto (PT) - Temporário</t>
-  </si>
-  <si>
-    <t>Operador ajudante do 1</t>
-  </si>
-  <si>
-    <t>24982928 2AP13</t>
-  </si>
-  <si>
-    <t>Test_4</t>
-  </si>
-  <si>
     <t>PortugalFour</t>
   </si>
   <si>
-    <t>Auto 48303176</t>
+    <t>Auto 71477403</t>
   </si>
   <si>
     <t>Fixed Term (Fixed Term)</t>
@@ -453,6 +478,9 @@
     <t>Test_5</t>
   </si>
   <si>
+    <t>10697814</t>
+  </si>
+  <si>
     <t>PortugalFive</t>
   </si>
   <si>
@@ -474,10 +502,13 @@
     <t>Test_6</t>
   </si>
   <si>
+    <t>10697815</t>
+  </si>
+  <si>
     <t>PortugalSix</t>
   </si>
   <si>
-    <t>Auto 20359541</t>
+    <t>Auto 78633043</t>
   </si>
   <si>
     <t>P&amp;C Manager Stores</t>
@@ -492,6 +523,9 @@
     <t>Test_7</t>
   </si>
   <si>
+    <t>10697816</t>
+  </si>
+  <si>
     <t>PortugalSeven</t>
   </si>
   <si>
@@ -510,10 +544,13 @@
     <t>Test_8</t>
   </si>
   <si>
+    <t>10697817</t>
+  </si>
+  <si>
     <t>PortugalEight</t>
   </si>
   <si>
-    <t>Auto 73786272</t>
+    <t>Auto 62296187</t>
   </si>
   <si>
     <t>Trainee Manager</t>
@@ -525,6 +562,9 @@
     <t>Test_9</t>
   </si>
   <si>
+    <t>10697818</t>
+  </si>
+  <si>
     <t>PortugalNine</t>
   </si>
   <si>
@@ -540,10 +580,13 @@
     <t>Test_10</t>
   </si>
   <si>
+    <t>10697819</t>
+  </si>
+  <si>
     <t>PortugalTen</t>
   </si>
   <si>
-    <t>Auto 65858312</t>
+    <t>Auto 11474280</t>
   </si>
   <si>
     <t>Service Contract</t>
@@ -561,6 +604,9 @@
     <t>Test_11</t>
   </si>
   <si>
+    <t>10697820</t>
+  </si>
+  <si>
     <t>PortugalEleven</t>
   </si>
   <si>
@@ -570,10 +616,13 @@
     <t>Test_12</t>
   </si>
   <si>
+    <t>10697821</t>
+  </si>
+  <si>
     <t>PortugalTwelve</t>
   </si>
   <si>
-    <t>Auto 16490201</t>
+    <t>Auto 46638489</t>
   </si>
   <si>
     <t>Department Manager</t>
@@ -585,6 +634,9 @@
     <t>Test_13</t>
   </si>
   <si>
+    <t>10697822</t>
+  </si>
+  <si>
     <t>PortugalThirteen</t>
   </si>
   <si>
@@ -603,10 +655,13 @@
     <t>Test_14</t>
   </si>
   <si>
+    <t>10697824</t>
+  </si>
+  <si>
     <t>PortugalFourteen</t>
   </si>
   <si>
-    <t>Auto 58720018</t>
+    <t>Auto 48272921</t>
   </si>
   <si>
     <t>24982928 2AP24</t>
@@ -615,10 +670,13 @@
     <t>Test_15</t>
   </si>
   <si>
+    <t>10697825</t>
+  </si>
+  <si>
     <t>PortugalFifteen</t>
   </si>
   <si>
-    <t>Auto 15082024 100703 AM</t>
+    <t>Auto 53134627</t>
   </si>
   <si>
     <t>24982928 2AP25</t>
@@ -627,92 +685,92 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yyyy"/>
   </numFmts>
   <fonts count="12" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
+      <name val="Calibri Light"/>
       <family val="2"/>
       <scheme val="major"/>
-      <sz val="10"/>
-      <name val="Calibri Light"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color theme="1"/>
+      <name val="Calibri Light"/>
       <family val="2"/>
       <scheme val="major"/>
-      <sz val="10"/>
-      <name val="Calibri Light"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="10"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="11"/>
       <color indexed="8"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="14"/>
       <color theme="1"/>
+      <name val="Arial"/>
       <family val="2"/>
-      <sz val="14"/>
-      <name val="Arial"/>
     </font>
     <font>
+      <sz val="11"/>
       <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <u/>
+      <sz val="11"/>
       <color indexed="12"/>
+      <name val="Calibri"/>
       <family val="2"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
       <u/>
+      <sz val="11"/>
       <color theme="10"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
     <font>
+      <sz val="7"/>
       <color rgb="FF1F1F1F"/>
+      <name val="Courier New"/>
       <family val="3"/>
-      <sz val="7"/>
-      <name val="Courier New"/>
     </font>
     <font>
+      <sz val="10"/>
       <color indexed="8"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="10"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="8">
@@ -735,7 +793,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="0" tint="-0.1499984740745262"/>
+        <fgColor theme="0" tint="-0.14999847407452621"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -747,13 +805,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.7999816888943144"/>
-        <bgColor indexed="64"/>
+        <fgColor rgb="FF00FF00"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00FF00"/>
+        <fgColor theme="5" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -772,24 +830,42 @@
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -827,7 +903,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -836,7 +912,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -857,7 +933,7 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left"/>
       <protection locked="0"/>
     </xf>
@@ -907,7 +983,7 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1189,9 +1265,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:BZ76"/>
-  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
+  <sheetFormatPr defaultRowHeight="14.4" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.33203125" customWidth="1"/>
     <col min="2" max="2" width="11.109375" customWidth="1"/>
@@ -1271,7 +1347,7 @@
     <col min="77" max="77" width="22.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.4" customHeight="1" spans="1:67" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:77" s="2" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1474,7 +1550,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" ht="17.4" customHeight="1" spans="1:77" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:77" s="10" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
         <v>64</v>
       </c>
@@ -1509,8 +1585,8 @@
         <v>73</v>
       </c>
       <c r="L2" s="19">
-        <f t="shared" ref="L2:L16" si="0">TODAY()-31</f>
-        <v>45725</v>
+        <f t="shared" ref="L2:L16" ca="1" si="0">TODAY()-31</f>
+        <v>45726</v>
       </c>
       <c r="M2" s="14" t="s">
         <v>68</v>
@@ -1537,8 +1613,8 @@
         <v>73</v>
       </c>
       <c r="U2" s="19">
-        <f t="shared" ref="U2:U16" si="1">L2</f>
-        <v>45725</v>
+        <f t="shared" ref="U2:U16" ca="1" si="1">L2</f>
+        <v>45726</v>
       </c>
       <c r="V2" s="18" t="s">
         <v>79</v>
@@ -1589,12 +1665,12 @@
         <v>99</v>
       </c>
       <c r="AL2" s="21">
-        <f t="shared" ref="AL2:AL16" si="2">TODAY()+60</f>
-        <v>45816</v>
+        <f t="shared" ref="AL2:AL16" ca="1" si="2">TODAY()+60</f>
+        <v>45817</v>
       </c>
       <c r="AM2" s="21">
-        <f t="shared" ref="AM2:AM16" si="3">U2</f>
-        <v>45725</v>
+        <f t="shared" ref="AM2:AM16" ca="1" si="3">U2</f>
+        <v>45726</v>
       </c>
       <c r="AN2" s="29" t="s">
         <v>93</v>
@@ -1605,9 +1681,9 @@
       <c r="AP2" s="21" t="s">
         <v>95</v>
       </c>
-      <c r="AQ2" s="19">
+      <c r="AQ2" s="19" t="str">
         <f t="shared" ref="AQ2:AQ9" si="4">AE2</f>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AR2" s="14" t="s">
         <v>96</v>
@@ -1652,7 +1728,7 @@
         <v>104</v>
       </c>
       <c r="BF2" s="33">
-        <v>10000299514.5239</v>
+        <v>10000056640.381001</v>
       </c>
       <c r="BG2" s="32" t="s">
         <v>68</v>
@@ -1661,7 +1737,7 @@
         <v>105</v>
       </c>
       <c r="BI2" s="33">
-        <v>100249714.523806</v>
+        <v>100006840.38094699</v>
       </c>
       <c r="BJ2" s="32" t="s">
         <v>68</v>
@@ -1692,7 +1768,7 @@
       <c r="BX2" s="12"/>
       <c r="BY2" s="12"/>
     </row>
-    <row r="3" ht="17.4" customHeight="1" spans="1:77" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:77" s="10" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="36" t="s">
         <v>111</v>
       </c>
@@ -1700,19 +1776,19 @@
         <v>112</v>
       </c>
       <c r="C3" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="D3" s="13" t="s">
         <v>113</v>
       </c>
-      <c r="D3" s="13" t="s">
+      <c r="E3" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="F3" s="15" t="s">
         <v>114</v>
       </c>
-      <c r="E3" s="14" t="s">
-        <v>68</v>
-      </c>
-      <c r="F3" s="15" t="s">
+      <c r="G3" s="16" t="s">
         <v>115</v>
-      </c>
-      <c r="G3" s="16" t="s">
-        <v>70</v>
       </c>
       <c r="H3" s="17" t="s">
         <v>116</v>
@@ -1727,8 +1803,8 @@
         <v>73</v>
       </c>
       <c r="L3" s="19">
-        <f t="shared" si="0"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45726</v>
       </c>
       <c r="M3" s="14" t="s">
         <v>68</v>
@@ -1755,8 +1831,8 @@
         <v>73</v>
       </c>
       <c r="U3" s="19">
-        <f t="shared" si="1"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45726</v>
       </c>
       <c r="V3" s="18" t="s">
         <v>117</v>
@@ -1807,12 +1883,12 @@
         <v>99</v>
       </c>
       <c r="AL3" s="21">
-        <f t="shared" si="2"/>
-        <v>45816</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45817</v>
       </c>
       <c r="AM3" s="21">
-        <f t="shared" si="3"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45726</v>
       </c>
       <c r="AN3" s="29" t="s">
         <v>121</v>
@@ -1823,9 +1899,9 @@
       <c r="AP3" s="21" t="s">
         <v>95</v>
       </c>
-      <c r="AQ3" s="19">
+      <c r="AQ3" s="19" t="str">
         <f t="shared" si="4"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AR3" s="14" t="s">
         <v>96</v>
@@ -1870,7 +1946,7 @@
         <v>104</v>
       </c>
       <c r="BF3" s="33">
-        <v>10000285227.8096</v>
+        <v>10000070927.095301</v>
       </c>
       <c r="BG3" s="32" t="s">
         <v>68</v>
@@ -1879,7 +1955,7 @@
         <v>105</v>
       </c>
       <c r="BI3" s="33">
-        <v>100235427.80952</v>
+        <v>100021127.09523299</v>
       </c>
       <c r="BJ3" s="32" t="s">
         <v>68</v>
@@ -1910,12 +1986,16 @@
       <c r="BX3" s="12"/>
       <c r="BY3" s="12"/>
     </row>
-    <row r="4" ht="17.4" customHeight="1" spans="1:77" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:77" s="10" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="36" t="s">
         <v>125</v>
       </c>
-      <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
+      <c r="B4" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="C4" s="12" t="s">
+        <v>66</v>
+      </c>
       <c r="D4" s="13" t="s">
         <v>67</v>
       </c>
@@ -1923,10 +2003,10 @@
         <v>68</v>
       </c>
       <c r="F4" s="15" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="G4" s="16" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="H4" s="17" t="s">
         <v>71</v>
@@ -1941,8 +2021,8 @@
         <v>73</v>
       </c>
       <c r="L4" s="19">
-        <f t="shared" si="0"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45726</v>
       </c>
       <c r="M4" s="14" t="s">
         <v>68</v>
@@ -1969,8 +2049,8 @@
         <v>73</v>
       </c>
       <c r="U4" s="19">
-        <f t="shared" si="1"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45726</v>
       </c>
       <c r="V4" s="18" t="s">
         <v>79</v>
@@ -1979,13 +2059,13 @@
         <v>80</v>
       </c>
       <c r="X4" s="21" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="Y4" s="24" t="s">
         <v>82</v>
       </c>
       <c r="Z4" s="21" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="AA4" s="25" t="s">
         <v>84</v>
@@ -2000,14 +2080,14 @@
         <v>86</v>
       </c>
       <c r="AE4" s="19">
-        <f>TODAY()+365</f>
-        <v>46121</v>
+        <f ca="1">TODAY()+365</f>
+        <v>46122</v>
       </c>
       <c r="AF4" s="18" t="s">
         <v>88</v>
       </c>
       <c r="AG4" s="27" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="AH4" s="18" t="s">
         <v>90</v>
@@ -2022,25 +2102,25 @@
         <v>99</v>
       </c>
       <c r="AL4" s="21">
-        <f t="shared" si="2"/>
-        <v>45816</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45817</v>
       </c>
       <c r="AM4" s="21">
-        <f t="shared" si="3"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45726</v>
       </c>
       <c r="AN4" s="29" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="AO4" s="20" t="s">
         <v>94</v>
       </c>
       <c r="AP4" s="21" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="AQ4" s="19">
-        <f t="shared" si="4"/>
-        <v>46121</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46122</v>
       </c>
       <c r="AR4" s="14" t="s">
         <v>96</v>
@@ -2049,7 +2129,7 @@
         <v>97</v>
       </c>
       <c r="AT4" s="14" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="AU4" s="14" t="s">
         <v>96</v>
@@ -2085,7 +2165,7 @@
         <v>104</v>
       </c>
       <c r="BF4" s="33">
-        <v>10000270941.0953</v>
+        <v>10000270941.095301</v>
       </c>
       <c r="BG4" s="32" t="s">
         <v>68</v>
@@ -2094,7 +2174,7 @@
         <v>105</v>
       </c>
       <c r="BI4" s="33">
-        <v>100221141.095234</v>
+        <v>100221141.09523401</v>
       </c>
       <c r="BJ4" s="32" t="s">
         <v>68</v>
@@ -2103,7 +2183,7 @@
         <v>106</v>
       </c>
       <c r="BL4" s="35" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="BM4" s="32" t="s">
         <v>108</v>
@@ -2125,23 +2205,27 @@
       <c r="BX4" s="12"/>
       <c r="BY4" s="12"/>
     </row>
-    <row r="5" ht="17.4" customHeight="1" spans="1:77" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:77" s="10" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="36" t="s">
-        <v>134</v>
-      </c>
-      <c r="B5" s="37"/>
-      <c r="C5" s="12"/>
+        <v>136</v>
+      </c>
+      <c r="B5" s="37" t="s">
+        <v>137</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>138</v>
+      </c>
       <c r="D5" s="13" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E5" s="14" t="s">
         <v>68</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="H5" s="17" t="s">
         <v>116</v>
@@ -2156,8 +2240,8 @@
         <v>73</v>
       </c>
       <c r="L5" s="19">
-        <f t="shared" si="0"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45726</v>
       </c>
       <c r="M5" s="14" t="s">
         <v>68</v>
@@ -2184,20 +2268,20 @@
         <v>73</v>
       </c>
       <c r="U5" s="19">
-        <f t="shared" si="1"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45726</v>
       </c>
       <c r="V5" s="18" t="s">
         <v>117</v>
       </c>
       <c r="W5" s="23" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="X5" s="39" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="Y5" s="24" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="Z5" s="21" t="s">
         <v>83</v>
@@ -2215,8 +2299,8 @@
         <v>86</v>
       </c>
       <c r="AE5" s="19">
-        <f>TODAY()+365</f>
-        <v>46121</v>
+        <f ca="1">TODAY()+365</f>
+        <v>46122</v>
       </c>
       <c r="AF5" s="18" t="s">
         <v>120</v>
@@ -2237,25 +2321,25 @@
         <v>99</v>
       </c>
       <c r="AL5" s="21">
-        <f t="shared" si="2"/>
-        <v>45816</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45817</v>
       </c>
       <c r="AM5" s="21">
-        <f t="shared" si="3"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45726</v>
       </c>
       <c r="AN5" s="29" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="AO5" s="20" t="s">
         <v>94</v>
       </c>
       <c r="AP5" s="21" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="AQ5" s="19">
-        <f t="shared" si="4"/>
-        <v>46121</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46122</v>
       </c>
       <c r="AR5" s="14" t="s">
         <v>96</v>
@@ -2300,7 +2384,7 @@
         <v>104</v>
       </c>
       <c r="BF5" s="33">
-        <v>10000256654.381</v>
+        <v>10000256654.381001</v>
       </c>
       <c r="BG5" s="32" t="s">
         <v>68</v>
@@ -2309,7 +2393,7 @@
         <v>105</v>
       </c>
       <c r="BI5" s="33">
-        <v>100206854.380948</v>
+        <v>100206854.38094801</v>
       </c>
       <c r="BJ5" s="32" t="s">
         <v>68</v>
@@ -2318,7 +2402,7 @@
         <v>106</v>
       </c>
       <c r="BL5" s="35" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="BM5" s="32" t="s">
         <v>108</v>
@@ -2340,12 +2424,16 @@
       <c r="BX5" s="12"/>
       <c r="BY5" s="12"/>
     </row>
-    <row r="6" ht="17.4" customHeight="1" spans="1:77" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:77" s="10" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="36" t="s">
-        <v>142</v>
-      </c>
-      <c r="B6" s="12"/>
-      <c r="C6" s="12"/>
+        <v>146</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>147</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>66</v>
+      </c>
       <c r="D6" s="13" t="s">
         <v>67</v>
       </c>
@@ -2353,10 +2441,10 @@
         <v>68</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="G6" s="16" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="H6" s="17" t="s">
         <v>71</v>
@@ -2371,8 +2459,8 @@
         <v>73</v>
       </c>
       <c r="L6" s="19">
-        <f t="shared" si="0"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45726</v>
       </c>
       <c r="M6" s="14" t="s">
         <v>68</v>
@@ -2399,8 +2487,8 @@
         <v>73</v>
       </c>
       <c r="U6" s="19">
-        <f t="shared" si="1"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45726</v>
       </c>
       <c r="V6" s="18" t="s">
         <v>79</v>
@@ -2412,7 +2500,7 @@
         <v>81</v>
       </c>
       <c r="Y6" s="24" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="Z6" s="21" t="s">
         <v>83</v>
@@ -2436,7 +2524,7 @@
         <v>88</v>
       </c>
       <c r="AG6" s="10" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="AH6" s="18" t="s">
         <v>90</v>
@@ -2451,15 +2539,15 @@
         <v>99</v>
       </c>
       <c r="AL6" s="21">
-        <f t="shared" si="2"/>
-        <v>45816</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45817</v>
       </c>
       <c r="AM6" s="21">
-        <f t="shared" si="3"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45726</v>
       </c>
       <c r="AN6" s="29" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="AO6" s="20" t="s">
         <v>94</v>
@@ -2467,15 +2555,15 @@
       <c r="AP6" s="21" t="s">
         <v>95</v>
       </c>
-      <c r="AQ6" s="19">
+      <c r="AQ6" s="19" t="str">
         <f t="shared" si="4"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AR6" s="14" t="s">
         <v>96</v>
       </c>
       <c r="AS6" s="14" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="AT6" s="14" t="s">
         <v>87</v>
@@ -2523,7 +2611,7 @@
         <v>105</v>
       </c>
       <c r="BI6" s="33">
-        <v>100192567.666662</v>
+        <v>100192567.66666199</v>
       </c>
       <c r="BJ6" s="32" t="s">
         <v>68</v>
@@ -2532,7 +2620,7 @@
         <v>106</v>
       </c>
       <c r="BL6" s="35" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="BM6" s="32" t="s">
         <v>108</v>
@@ -2554,23 +2642,27 @@
       <c r="BX6" s="12"/>
       <c r="BY6" s="12"/>
     </row>
-    <row r="7" ht="17.4" customHeight="1" spans="1:77" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:77" s="10" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="36" t="s">
-        <v>149</v>
-      </c>
-      <c r="B7" s="40"/>
-      <c r="C7" s="12"/>
+        <v>154</v>
+      </c>
+      <c r="B7" s="40" t="s">
+        <v>155</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>66</v>
+      </c>
       <c r="D7" s="13" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E7" s="14" t="s">
         <v>68</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="H7" s="17" t="s">
         <v>116</v>
@@ -2585,8 +2677,8 @@
         <v>73</v>
       </c>
       <c r="L7" s="19">
-        <f t="shared" si="0"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45726</v>
       </c>
       <c r="M7" s="14" t="s">
         <v>68</v>
@@ -2613,23 +2705,23 @@
         <v>73</v>
       </c>
       <c r="U7" s="19">
-        <f t="shared" si="1"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45726</v>
       </c>
       <c r="V7" s="18" t="s">
         <v>79</v>
       </c>
       <c r="W7" s="23" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="X7" s="21" t="s">
         <v>81</v>
       </c>
       <c r="Y7" s="24" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="Z7" s="21" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="AA7" s="25" t="s">
         <v>84</v>
@@ -2665,15 +2757,15 @@
         <v>99</v>
       </c>
       <c r="AL7" s="21">
-        <f t="shared" si="2"/>
-        <v>45816</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45817</v>
       </c>
       <c r="AM7" s="21">
-        <f t="shared" si="3"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45726</v>
       </c>
       <c r="AN7" s="29" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="AO7" s="20" t="s">
         <v>94</v>
@@ -2681,9 +2773,9 @@
       <c r="AP7" s="21" t="s">
         <v>95</v>
       </c>
-      <c r="AQ7" s="19">
+      <c r="AQ7" s="19" t="str">
         <f t="shared" si="4"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AR7" s="14" t="s">
         <v>96</v>
@@ -2737,7 +2829,7 @@
         <v>105</v>
       </c>
       <c r="BI7" s="33">
-        <v>100178280.952376</v>
+        <v>100178280.95237599</v>
       </c>
       <c r="BJ7" s="32" t="s">
         <v>68</v>
@@ -2746,7 +2838,7 @@
         <v>106</v>
       </c>
       <c r="BL7" s="35" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="BM7" s="32" t="s">
         <v>108</v>
@@ -2768,12 +2860,16 @@
       <c r="BX7" s="12"/>
       <c r="BY7" s="12"/>
     </row>
-    <row r="8" ht="17.4" customHeight="1" spans="1:77" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:77" s="10" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="36" t="s">
-        <v>155</v>
-      </c>
-      <c r="B8" s="37"/>
-      <c r="C8" s="12"/>
+        <v>161</v>
+      </c>
+      <c r="B8" s="37" t="s">
+        <v>162</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>66</v>
+      </c>
       <c r="D8" s="13" t="s">
         <v>67</v>
       </c>
@@ -2781,10 +2877,10 @@
         <v>68</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="G8" s="16" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="H8" s="17" t="s">
         <v>71</v>
@@ -2799,8 +2895,8 @@
         <v>73</v>
       </c>
       <c r="L8" s="19">
-        <f t="shared" si="0"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45726</v>
       </c>
       <c r="M8" s="14" t="s">
         <v>68</v>
@@ -2827,8 +2923,8 @@
         <v>73</v>
       </c>
       <c r="U8" s="19">
-        <f t="shared" si="1"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45726</v>
       </c>
       <c r="V8" s="18" t="s">
         <v>79</v>
@@ -2837,13 +2933,13 @@
         <v>80</v>
       </c>
       <c r="X8" s="39" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="Y8" s="24" t="s">
         <v>82</v>
       </c>
       <c r="Z8" s="21" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="AA8" s="25" t="s">
         <v>84</v>
@@ -2855,11 +2951,11 @@
         <v>85</v>
       </c>
       <c r="AD8" s="14" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="AE8" s="19">
-        <f>TODAY()+365</f>
-        <v>46121</v>
+        <f ca="1">TODAY()+365</f>
+        <v>46122</v>
       </c>
       <c r="AF8" s="18" t="s">
         <v>88</v>
@@ -2880,25 +2976,25 @@
         <v>99</v>
       </c>
       <c r="AL8" s="21">
-        <f t="shared" si="2"/>
-        <v>45816</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45817</v>
       </c>
       <c r="AM8" s="21">
-        <f t="shared" si="3"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45726</v>
       </c>
       <c r="AN8" s="29" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="AO8" s="20" t="s">
         <v>94</v>
       </c>
       <c r="AP8" s="21" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="AQ8" s="19">
-        <f t="shared" si="4"/>
-        <v>46121</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46122</v>
       </c>
       <c r="AR8" s="14" t="s">
         <v>96</v>
@@ -2907,7 +3003,7 @@
         <v>97</v>
       </c>
       <c r="AT8" s="14" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="AU8" s="14" t="s">
         <v>96</v>
@@ -2952,7 +3048,7 @@
         <v>105</v>
       </c>
       <c r="BI8" s="33">
-        <v>100163994.23809</v>
+        <v>100163994.23808999</v>
       </c>
       <c r="BJ8" s="32" t="s">
         <v>68</v>
@@ -2961,7 +3057,7 @@
         <v>106</v>
       </c>
       <c r="BL8" s="35" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="BM8" s="32" t="s">
         <v>108</v>
@@ -2983,23 +3079,27 @@
       <c r="BX8" s="12"/>
       <c r="BY8" s="12"/>
     </row>
-    <row r="9" ht="17.4" customHeight="1" spans="1:77" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:77" s="10" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="36" t="s">
-        <v>161</v>
-      </c>
-      <c r="B9" s="12"/>
-      <c r="C9" s="12"/>
+        <v>168</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>66</v>
+      </c>
       <c r="D9" s="13" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E9" s="14" t="s">
         <v>68</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="H9" s="17" t="s">
         <v>116</v>
@@ -3014,8 +3114,8 @@
         <v>73</v>
       </c>
       <c r="L9" s="19">
-        <f t="shared" si="0"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45726</v>
       </c>
       <c r="M9" s="14" t="s">
         <v>68</v>
@@ -3042,20 +3142,20 @@
         <v>73</v>
       </c>
       <c r="U9" s="19">
-        <f t="shared" si="1"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45726</v>
       </c>
       <c r="V9" s="18" t="s">
         <v>79</v>
       </c>
       <c r="W9" s="23" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="X9" s="39" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="Y9" s="24" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="Z9" s="21" t="s">
         <v>83</v>
@@ -3073,8 +3173,8 @@
         <v>86</v>
       </c>
       <c r="AE9" s="19">
-        <f>TODAY()+365</f>
-        <v>46121</v>
+        <f ca="1">TODAY()+365</f>
+        <v>46122</v>
       </c>
       <c r="AF9" s="18" t="s">
         <v>120</v>
@@ -3095,12 +3195,12 @@
         <v>99</v>
       </c>
       <c r="AL9" s="21">
-        <f t="shared" si="2"/>
-        <v>45816</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45817</v>
       </c>
       <c r="AM9" s="21">
-        <f t="shared" si="3"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45726</v>
       </c>
       <c r="AN9" s="29" t="s">
         <v>93</v>
@@ -3109,11 +3209,11 @@
         <v>94</v>
       </c>
       <c r="AP9" s="21" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="AQ9" s="19">
-        <f t="shared" si="4"/>
-        <v>46121</v>
+        <f t="shared" ca="1" si="4"/>
+        <v>46122</v>
       </c>
       <c r="AR9" s="14" t="s">
         <v>96</v>
@@ -3158,7 +3258,7 @@
         <v>104</v>
       </c>
       <c r="BF9" s="33">
-        <v>10000199507.5239</v>
+        <v>10000199507.523899</v>
       </c>
       <c r="BG9" s="32" t="s">
         <v>68</v>
@@ -3167,7 +3267,7 @@
         <v>105</v>
       </c>
       <c r="BI9" s="33">
-        <v>100149707.523804</v>
+        <v>100149707.52380399</v>
       </c>
       <c r="BJ9" s="32" t="s">
         <v>68</v>
@@ -3176,7 +3276,7 @@
         <v>106</v>
       </c>
       <c r="BL9" s="35" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
       <c r="BM9" s="32" t="s">
         <v>108</v>
@@ -3198,12 +3298,16 @@
       <c r="BX9" s="12"/>
       <c r="BY9" s="12"/>
     </row>
-    <row r="10" ht="17.4" customHeight="1" spans="1:77" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:77" s="10" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="36" t="s">
-        <v>166</v>
-      </c>
-      <c r="B10" s="12"/>
-      <c r="C10" s="12"/>
+        <v>174</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>175</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>66</v>
+      </c>
       <c r="D10" s="13" t="s">
         <v>67</v>
       </c>
@@ -3211,10 +3315,10 @@
         <v>68</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
       <c r="G10" s="16" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="H10" s="17" t="s">
         <v>71</v>
@@ -3229,8 +3333,8 @@
         <v>73</v>
       </c>
       <c r="L10" s="19">
-        <f t="shared" si="0"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45726</v>
       </c>
       <c r="M10" s="14" t="s">
         <v>68</v>
@@ -3257,8 +3361,8 @@
         <v>73</v>
       </c>
       <c r="U10" s="19">
-        <f t="shared" si="1"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45726</v>
       </c>
       <c r="V10" s="18" t="s">
         <v>79</v>
@@ -3267,7 +3371,7 @@
         <v>80</v>
       </c>
       <c r="X10" s="21" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="Y10" s="24" t="s">
         <v>82</v>
@@ -3294,7 +3398,7 @@
         <v>88</v>
       </c>
       <c r="AG10" s="27" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="AH10" s="18" t="s">
         <v>90</v>
@@ -3309,12 +3413,12 @@
         <v>99</v>
       </c>
       <c r="AL10" s="21">
-        <f t="shared" si="2"/>
-        <v>45816</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45817</v>
       </c>
       <c r="AM10" s="21">
-        <f t="shared" si="3"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45726</v>
       </c>
       <c r="AN10" s="29" t="s">
         <v>121</v>
@@ -3323,11 +3427,11 @@
         <v>94</v>
       </c>
       <c r="AP10" s="21" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="AQ10" s="19">
-        <f>U10+365</f>
-        <v>46090</v>
+        <f ca="1">U10+365</f>
+        <v>46091</v>
       </c>
       <c r="AR10" s="14" t="s">
         <v>96</v>
@@ -3336,7 +3440,7 @@
         <v>97</v>
       </c>
       <c r="AT10" s="14" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="AU10" s="14" t="s">
         <v>96</v>
@@ -3372,7 +3476,7 @@
         <v>104</v>
       </c>
       <c r="BF10" s="33">
-        <v>10000185220.8096</v>
+        <v>10000185220.809601</v>
       </c>
       <c r="BG10" s="32" t="s">
         <v>68</v>
@@ -3381,7 +3485,7 @@
         <v>105</v>
       </c>
       <c r="BI10" s="33">
-        <v>100135420.809518</v>
+        <v>100135420.80951799</v>
       </c>
       <c r="BJ10" s="32" t="s">
         <v>68</v>
@@ -3390,7 +3494,7 @@
         <v>106</v>
       </c>
       <c r="BL10" s="35" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="BM10" s="32" t="s">
         <v>108</v>
@@ -3412,23 +3516,27 @@
       <c r="BX10" s="12"/>
       <c r="BY10" s="12"/>
     </row>
-    <row r="11" ht="17.4" customHeight="1" spans="1:77" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:77" s="10" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="36" t="s">
-        <v>171</v>
-      </c>
-      <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
+        <v>180</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>181</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>66</v>
+      </c>
       <c r="D11" s="13" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E11" s="14" t="s">
         <v>68</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>172</v>
+        <v>182</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="H11" s="17" t="s">
         <v>116</v>
@@ -3443,8 +3551,8 @@
         <v>73</v>
       </c>
       <c r="L11" s="19">
-        <f t="shared" si="0"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45726</v>
       </c>
       <c r="M11" s="14" t="s">
         <v>68</v>
@@ -3471,23 +3579,23 @@
         <v>73</v>
       </c>
       <c r="U11" s="19">
-        <f t="shared" si="1"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45726</v>
       </c>
       <c r="V11" s="18" t="s">
         <v>79</v>
       </c>
       <c r="W11" s="23" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="X11" s="21" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
       <c r="Y11" s="24" t="s">
-        <v>175</v>
+        <v>185</v>
       </c>
       <c r="Z11" s="21" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="AA11" s="25" t="s">
         <v>84</v>
@@ -3523,25 +3631,25 @@
         <v>99</v>
       </c>
       <c r="AL11" s="21">
-        <f t="shared" si="2"/>
-        <v>45816</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45817</v>
       </c>
       <c r="AM11" s="21">
-        <f t="shared" si="3"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45726</v>
       </c>
       <c r="AN11" s="29" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="AO11" s="20" t="s">
         <v>94</v>
       </c>
       <c r="AP11" s="21" t="s">
-        <v>176</v>
-      </c>
-      <c r="AQ11" s="19">
+        <v>186</v>
+      </c>
+      <c r="AQ11" s="19" t="str">
         <f t="shared" ref="AQ11:AQ16" si="5">AE11</f>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AR11" s="14" t="s">
         <v>96</v>
@@ -3586,7 +3694,7 @@
         <v>104</v>
       </c>
       <c r="BF11" s="33">
-        <v>10000170934.0953</v>
+        <v>10000170934.095301</v>
       </c>
       <c r="BG11" s="32" t="s">
         <v>68</v>
@@ -3595,7 +3703,7 @@
         <v>105</v>
       </c>
       <c r="BI11" s="33">
-        <v>100121134.095232</v>
+        <v>100121134.09523199</v>
       </c>
       <c r="BJ11" s="32" t="s">
         <v>68</v>
@@ -3604,7 +3712,7 @@
         <v>106</v>
       </c>
       <c r="BL11" s="35" t="s">
-        <v>177</v>
+        <v>187</v>
       </c>
       <c r="BM11" s="32" t="s">
         <v>108</v>
@@ -3626,12 +3734,16 @@
       <c r="BX11" s="12"/>
       <c r="BY11" s="12"/>
     </row>
-    <row r="12" ht="17.4" customHeight="1" spans="1:77" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:77" s="10" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="36" t="s">
-        <v>178</v>
-      </c>
-      <c r="B12" s="12"/>
-      <c r="C12" s="12"/>
+        <v>188</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>189</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>66</v>
+      </c>
       <c r="D12" s="13" t="s">
         <v>67</v>
       </c>
@@ -3639,10 +3751,10 @@
         <v>68</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="G12" s="16" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="H12" s="17" t="s">
         <v>71</v>
@@ -3657,8 +3769,8 @@
         <v>73</v>
       </c>
       <c r="L12" s="19">
-        <f t="shared" si="0"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45726</v>
       </c>
       <c r="M12" s="14" t="s">
         <v>68</v>
@@ -3685,8 +3797,8 @@
         <v>73</v>
       </c>
       <c r="U12" s="19">
-        <f t="shared" si="1"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45726</v>
       </c>
       <c r="V12" s="18" t="s">
         <v>79</v>
@@ -3695,7 +3807,7 @@
         <v>80</v>
       </c>
       <c r="X12" s="21" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="Y12" s="24" t="s">
         <v>82</v>
@@ -3716,8 +3828,8 @@
         <v>86</v>
       </c>
       <c r="AE12" s="19">
-        <f>U12+365</f>
-        <v>46090</v>
+        <f ca="1">U12+365</f>
+        <v>46091</v>
       </c>
       <c r="AF12" s="18" t="s">
         <v>88</v>
@@ -3738,25 +3850,25 @@
         <v>99</v>
       </c>
       <c r="AL12" s="21">
-        <f t="shared" si="2"/>
-        <v>45816</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45817</v>
       </c>
       <c r="AM12" s="21">
-        <f t="shared" si="3"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45726</v>
       </c>
       <c r="AN12" s="29" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="AO12" s="20" t="s">
         <v>94</v>
       </c>
       <c r="AP12" s="21" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="AQ12" s="19">
-        <f t="shared" si="5"/>
-        <v>46090</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>46091</v>
       </c>
       <c r="AR12" s="14" t="s">
         <v>96</v>
@@ -3765,7 +3877,7 @@
         <v>97</v>
       </c>
       <c r="AT12" s="14" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="AU12" s="14" t="s">
         <v>96</v>
@@ -3801,7 +3913,7 @@
         <v>104</v>
       </c>
       <c r="BF12" s="33">
-        <v>10000156647.381</v>
+        <v>10000156647.381001</v>
       </c>
       <c r="BG12" s="32" t="s">
         <v>68</v>
@@ -3819,7 +3931,7 @@
         <v>106</v>
       </c>
       <c r="BL12" s="35" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="BM12" s="32" t="s">
         <v>108</v>
@@ -3841,23 +3953,27 @@
       <c r="BX12" s="12"/>
       <c r="BY12" s="12"/>
     </row>
-    <row r="13" ht="17.4" customHeight="1" spans="1:77" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:77" s="10" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="36" t="s">
-        <v>181</v>
-      </c>
-      <c r="B13" s="37"/>
-      <c r="C13" s="12"/>
+        <v>192</v>
+      </c>
+      <c r="B13" s="37" t="s">
+        <v>193</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>66</v>
+      </c>
       <c r="D13" s="13" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E13" s="14" t="s">
         <v>68</v>
       </c>
       <c r="F13" s="15" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="H13" s="17" t="s">
         <v>116</v>
@@ -3872,8 +3988,8 @@
         <v>73</v>
       </c>
       <c r="L13" s="19">
-        <f t="shared" si="0"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45726</v>
       </c>
       <c r="M13" s="14" t="s">
         <v>68</v>
@@ -3900,20 +4016,20 @@
         <v>73</v>
       </c>
       <c r="U13" s="19">
-        <f t="shared" si="1"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45726</v>
       </c>
       <c r="V13" s="18" t="s">
         <v>79</v>
       </c>
       <c r="W13" s="23" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="X13" s="39" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="Y13" s="24" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="Z13" s="21" t="s">
         <v>83</v>
@@ -3931,8 +4047,8 @@
         <v>86</v>
       </c>
       <c r="AE13" s="19">
-        <f>TODAY()+365</f>
-        <v>46121</v>
+        <f ca="1">TODAY()+365</f>
+        <v>46122</v>
       </c>
       <c r="AF13" s="18" t="s">
         <v>120</v>
@@ -3953,25 +4069,25 @@
         <v>99</v>
       </c>
       <c r="AL13" s="21">
-        <f t="shared" si="2"/>
-        <v>45816</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45817</v>
       </c>
       <c r="AM13" s="21">
-        <f t="shared" si="3"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45726</v>
       </c>
       <c r="AN13" s="29" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="AO13" s="20" t="s">
         <v>94</v>
       </c>
       <c r="AP13" s="21" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="AQ13" s="19">
-        <f t="shared" si="5"/>
-        <v>46121</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>46122</v>
       </c>
       <c r="AR13" s="14" t="s">
         <v>96</v>
@@ -4034,7 +4150,7 @@
         <v>106</v>
       </c>
       <c r="BL13" s="35" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
       <c r="BM13" s="32" t="s">
         <v>108</v>
@@ -4056,12 +4172,16 @@
       <c r="BX13" s="12"/>
       <c r="BY13" s="12"/>
     </row>
-    <row r="14" ht="17.4" customHeight="1" spans="1:77" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:77" s="10" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="36" t="s">
-        <v>186</v>
-      </c>
-      <c r="B14" s="12"/>
-      <c r="C14" s="12"/>
+        <v>198</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>199</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>66</v>
+      </c>
       <c r="D14" s="13" t="s">
         <v>67</v>
       </c>
@@ -4069,10 +4189,10 @@
         <v>68</v>
       </c>
       <c r="F14" s="15" t="s">
-        <v>187</v>
+        <v>200</v>
       </c>
       <c r="G14" s="16" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="H14" s="17" t="s">
         <v>71</v>
@@ -4087,8 +4207,8 @@
         <v>73</v>
       </c>
       <c r="L14" s="19">
-        <f t="shared" si="0"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45726</v>
       </c>
       <c r="M14" s="14" t="s">
         <v>68</v>
@@ -4115,8 +4235,8 @@
         <v>73</v>
       </c>
       <c r="U14" s="19">
-        <f t="shared" si="1"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45726</v>
       </c>
       <c r="V14" s="18" t="s">
         <v>79</v>
@@ -4131,7 +4251,7 @@
         <v>82</v>
       </c>
       <c r="Z14" s="21" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="AA14" s="25" t="s">
         <v>84</v>
@@ -4143,7 +4263,7 @@
         <v>85</v>
       </c>
       <c r="AD14" s="14" t="s">
-        <v>188</v>
+        <v>201</v>
       </c>
       <c r="AE14" s="19" t="s">
         <v>87</v>
@@ -4152,7 +4272,7 @@
         <v>88</v>
       </c>
       <c r="AG14" s="27" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="AH14" s="18" t="s">
         <v>90</v>
@@ -4167,25 +4287,25 @@
         <v>99</v>
       </c>
       <c r="AL14" s="21">
-        <f t="shared" si="2"/>
-        <v>45816</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45817</v>
       </c>
       <c r="AM14" s="21">
-        <f t="shared" si="3"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45726</v>
       </c>
       <c r="AN14" s="29" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="AO14" s="20" t="s">
         <v>94</v>
       </c>
       <c r="AP14" s="21" t="s">
-        <v>189</v>
-      </c>
-      <c r="AQ14" s="19">
+        <v>202</v>
+      </c>
+      <c r="AQ14" s="19" t="str">
         <f t="shared" si="5"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AR14" s="14" t="s">
         <v>96</v>
@@ -4194,7 +4314,7 @@
         <v>97</v>
       </c>
       <c r="AT14" s="14" t="s">
-        <v>190</v>
+        <v>203</v>
       </c>
       <c r="AU14" s="14" t="s">
         <v>96</v>
@@ -4248,7 +4368,7 @@
         <v>106</v>
       </c>
       <c r="BL14" s="35" t="s">
-        <v>191</v>
+        <v>204</v>
       </c>
       <c r="BM14" s="32" t="s">
         <v>108</v>
@@ -4270,23 +4390,27 @@
       <c r="BX14" s="12"/>
       <c r="BY14" s="12"/>
     </row>
-    <row r="15" ht="17.4" customHeight="1" spans="1:77" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:77" s="10" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="36" t="s">
-        <v>192</v>
-      </c>
-      <c r="B15" s="37"/>
-      <c r="C15" s="12"/>
+        <v>205</v>
+      </c>
+      <c r="B15" s="37" t="s">
+        <v>206</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>66</v>
+      </c>
       <c r="D15" s="13" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E15" s="14" t="s">
         <v>68</v>
       </c>
       <c r="F15" s="15" t="s">
-        <v>193</v>
+        <v>207</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="H15" s="17" t="s">
         <v>116</v>
@@ -4301,8 +4425,8 @@
         <v>73</v>
       </c>
       <c r="L15" s="19">
-        <f t="shared" si="0"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45726</v>
       </c>
       <c r="M15" s="14" t="s">
         <v>68</v>
@@ -4329,23 +4453,23 @@
         <v>73</v>
       </c>
       <c r="U15" s="19">
-        <f t="shared" si="1"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45726</v>
       </c>
       <c r="V15" s="18" t="s">
         <v>79</v>
       </c>
       <c r="W15" s="23" t="s">
-        <v>194</v>
+        <v>208</v>
       </c>
       <c r="X15" s="21" t="s">
-        <v>174</v>
+        <v>184</v>
       </c>
       <c r="Y15" s="24" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="Z15" s="21" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="AA15" s="25" t="s">
         <v>84</v>
@@ -4381,25 +4505,25 @@
         <v>99</v>
       </c>
       <c r="AL15" s="21">
-        <f t="shared" si="2"/>
-        <v>45816</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45817</v>
       </c>
       <c r="AM15" s="21">
-        <f t="shared" si="3"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45726</v>
       </c>
       <c r="AN15" s="29" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
       <c r="AO15" s="20" t="s">
         <v>94</v>
       </c>
       <c r="AP15" s="21" t="s">
-        <v>176</v>
-      </c>
-      <c r="AQ15" s="19">
+        <v>186</v>
+      </c>
+      <c r="AQ15" s="19" t="str">
         <f t="shared" si="5"/>
-        <v>NaN</v>
+        <v>N/A</v>
       </c>
       <c r="AR15" s="14" t="s">
         <v>96</v>
@@ -4444,7 +4568,7 @@
         <v>104</v>
       </c>
       <c r="BF15" s="33">
-        <v>10000113787.2382</v>
+        <v>10000113787.238199</v>
       </c>
       <c r="BG15" s="32" t="s">
         <v>68</v>
@@ -4462,7 +4586,7 @@
         <v>106</v>
       </c>
       <c r="BL15" s="35" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="BM15" s="32" t="s">
         <v>108</v>
@@ -4484,23 +4608,27 @@
       <c r="BX15" s="12"/>
       <c r="BY15" s="12"/>
     </row>
-    <row r="16" ht="17.4" customHeight="1" spans="1:77" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:77" s="10" customFormat="1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="36" t="s">
-        <v>196</v>
-      </c>
-      <c r="B16" s="37"/>
-      <c r="C16" s="12"/>
+        <v>210</v>
+      </c>
+      <c r="B16" s="37" t="s">
+        <v>211</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>66</v>
+      </c>
       <c r="D16" s="13" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E16" s="14" t="s">
         <v>68</v>
       </c>
       <c r="F16" s="15" t="s">
-        <v>197</v>
+        <v>212</v>
       </c>
       <c r="G16" s="16" t="s">
-        <v>70</v>
+        <v>128</v>
       </c>
       <c r="H16" s="17" t="s">
         <v>71</v>
@@ -4515,8 +4643,8 @@
         <v>73</v>
       </c>
       <c r="L16" s="19">
-        <f t="shared" si="0"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="0"/>
+        <v>45726</v>
       </c>
       <c r="M16" s="14" t="s">
         <v>68</v>
@@ -4543,17 +4671,17 @@
         <v>73</v>
       </c>
       <c r="U16" s="19">
-        <f t="shared" si="1"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="1"/>
+        <v>45726</v>
       </c>
       <c r="V16" s="18" t="s">
         <v>79</v>
       </c>
       <c r="W16" s="23" t="s">
-        <v>198</v>
+        <v>213</v>
       </c>
       <c r="X16" s="21" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="Y16" s="24" t="s">
         <v>119</v>
@@ -4574,8 +4702,8 @@
         <v>86</v>
       </c>
       <c r="AE16" s="19">
-        <f>TODAY()+365</f>
-        <v>46121</v>
+        <f ca="1">TODAY()+365</f>
+        <v>46122</v>
       </c>
       <c r="AF16" s="18" t="s">
         <v>120</v>
@@ -4596,12 +4724,12 @@
         <v>99</v>
       </c>
       <c r="AL16" s="21">
-        <f t="shared" si="2"/>
-        <v>45816</v>
+        <f t="shared" ca="1" si="2"/>
+        <v>45817</v>
       </c>
       <c r="AM16" s="21">
-        <f t="shared" si="3"/>
-        <v>45725</v>
+        <f t="shared" ca="1" si="3"/>
+        <v>45726</v>
       </c>
       <c r="AN16" s="29" t="s">
         <v>93</v>
@@ -4610,11 +4738,11 @@
         <v>94</v>
       </c>
       <c r="AP16" s="21" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="AQ16" s="19">
-        <f t="shared" si="5"/>
-        <v>46121</v>
+        <f t="shared" ca="1" si="5"/>
+        <v>46122</v>
       </c>
       <c r="AR16" s="14" t="s">
         <v>96</v>
@@ -4659,7 +4787,7 @@
         <v>104</v>
       </c>
       <c r="BF16" s="33">
-        <v>10000099500.5239</v>
+        <v>10000099500.523899</v>
       </c>
       <c r="BG16" s="32" t="s">
         <v>68</v>
@@ -4677,7 +4805,7 @@
         <v>106</v>
       </c>
       <c r="BL16" s="35" t="s">
-        <v>199</v>
+        <v>214</v>
       </c>
       <c r="BM16" s="32" t="s">
         <v>108</v>
@@ -5659,7 +5787,7 @@
       <c r="BY28" s="12"/>
       <c r="BZ28" s="12"/>
     </row>
-    <row r="29" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A29" s="12"/>
       <c r="B29" s="12"/>
       <c r="C29" s="12"/>
@@ -5739,7 +5867,7 @@
       <c r="BY29" s="12"/>
       <c r="BZ29" s="12"/>
     </row>
-    <row r="30" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A30" s="12"/>
       <c r="B30" s="12"/>
       <c r="C30" s="12"/>
@@ -5819,7 +5947,7 @@
       <c r="BY30" s="12"/>
       <c r="BZ30" s="12"/>
     </row>
-    <row r="31" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A31" s="12"/>
       <c r="B31" s="12"/>
       <c r="C31" s="12"/>
@@ -5899,7 +6027,7 @@
       <c r="BY31" s="12"/>
       <c r="BZ31" s="12"/>
     </row>
-    <row r="32" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A32" s="12"/>
       <c r="B32" s="12"/>
       <c r="C32" s="12"/>
@@ -5979,7 +6107,7 @@
       <c r="BY32" s="12"/>
       <c r="BZ32" s="12"/>
     </row>
-    <row r="33" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A33" s="12"/>
       <c r="B33" s="12"/>
       <c r="C33" s="12"/>
@@ -6059,7 +6187,7 @@
       <c r="BY33" s="12"/>
       <c r="BZ33" s="12"/>
     </row>
-    <row r="34" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A34" s="12"/>
       <c r="B34" s="12"/>
       <c r="C34" s="12"/>
@@ -6139,7 +6267,7 @@
       <c r="BY34" s="12"/>
       <c r="BZ34" s="12"/>
     </row>
-    <row r="35" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A35" s="12"/>
       <c r="B35" s="12"/>
       <c r="C35" s="12"/>
@@ -6219,7 +6347,7 @@
       <c r="BY35" s="12"/>
       <c r="BZ35" s="12"/>
     </row>
-    <row r="36" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" s="12"/>
       <c r="B36" s="12"/>
       <c r="C36" s="12"/>
@@ -6299,7 +6427,7 @@
       <c r="BY36" s="12"/>
       <c r="BZ36" s="12"/>
     </row>
-    <row r="37" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A37" s="12"/>
       <c r="B37" s="12"/>
       <c r="C37" s="12"/>
@@ -6379,7 +6507,7 @@
       <c r="BY37" s="12"/>
       <c r="BZ37" s="12"/>
     </row>
-    <row r="38" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A38" s="12"/>
       <c r="B38" s="12"/>
       <c r="C38" s="12"/>
@@ -6459,7 +6587,7 @@
       <c r="BY38" s="12"/>
       <c r="BZ38" s="12"/>
     </row>
-    <row r="39" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A39" s="12"/>
       <c r="B39" s="12"/>
       <c r="C39" s="12"/>
@@ -6539,7 +6667,7 @@
       <c r="BY39" s="12"/>
       <c r="BZ39" s="12"/>
     </row>
-    <row r="40" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A40" s="12"/>
       <c r="B40" s="12"/>
       <c r="C40" s="12"/>
@@ -6619,7 +6747,7 @@
       <c r="BY40" s="12"/>
       <c r="BZ40" s="12"/>
     </row>
-    <row r="41" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A41" s="12"/>
       <c r="B41" s="12"/>
       <c r="C41" s="12"/>
@@ -6699,7 +6827,7 @@
       <c r="BY41" s="12"/>
       <c r="BZ41" s="12"/>
     </row>
-    <row r="42" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A42" s="12"/>
       <c r="B42" s="12"/>
       <c r="C42" s="12"/>
@@ -6779,7 +6907,7 @@
       <c r="BY42" s="12"/>
       <c r="BZ42" s="12"/>
     </row>
-    <row r="43" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A43" s="12"/>
       <c r="B43" s="12"/>
       <c r="C43" s="12"/>
@@ -6859,7 +6987,7 @@
       <c r="BY43" s="12"/>
       <c r="BZ43" s="12"/>
     </row>
-    <row r="44" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A44" s="12"/>
       <c r="B44" s="12"/>
       <c r="C44" s="12"/>
@@ -6939,7 +7067,7 @@
       <c r="BY44" s="12"/>
       <c r="BZ44" s="12"/>
     </row>
-    <row r="45" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A45" s="12"/>
       <c r="B45" s="12"/>
       <c r="C45" s="12"/>
@@ -7019,7 +7147,7 @@
       <c r="BY45" s="12"/>
       <c r="BZ45" s="12"/>
     </row>
-    <row r="46" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A46" s="12"/>
       <c r="B46" s="12"/>
       <c r="C46" s="12"/>
@@ -7099,7 +7227,7 @@
       <c r="BY46" s="12"/>
       <c r="BZ46" s="12"/>
     </row>
-    <row r="47" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A47" s="12"/>
       <c r="B47" s="12"/>
       <c r="C47" s="12"/>
@@ -7179,7 +7307,7 @@
       <c r="BY47" s="12"/>
       <c r="BZ47" s="12"/>
     </row>
-    <row r="48" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A48" s="12"/>
       <c r="B48" s="12"/>
       <c r="C48" s="12"/>
@@ -7259,7 +7387,7 @@
       <c r="BY48" s="12"/>
       <c r="BZ48" s="12"/>
     </row>
-    <row r="49" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A49" s="12"/>
       <c r="B49" s="12"/>
       <c r="C49" s="12"/>
@@ -7339,7 +7467,7 @@
       <c r="BY49" s="12"/>
       <c r="BZ49" s="12"/>
     </row>
-    <row r="50" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A50" s="12"/>
       <c r="B50" s="12"/>
       <c r="C50" s="12"/>
@@ -7419,7 +7547,7 @@
       <c r="BY50" s="12"/>
       <c r="BZ50" s="12"/>
     </row>
-    <row r="51" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A51" s="12"/>
       <c r="B51" s="12"/>
       <c r="C51" s="12"/>
@@ -7499,7 +7627,7 @@
       <c r="BY51" s="12"/>
       <c r="BZ51" s="12"/>
     </row>
-    <row r="52" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A52" s="12"/>
       <c r="B52" s="12"/>
       <c r="C52" s="12"/>
@@ -7579,7 +7707,7 @@
       <c r="BY52" s="12"/>
       <c r="BZ52" s="12"/>
     </row>
-    <row r="53" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:78" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A53" s="12"/>
       <c r="B53" s="12"/>
       <c r="C53" s="12"/>
@@ -7659,7 +7787,7 @@
       <c r="BY53" s="12"/>
       <c r="BZ53" s="12"/>
     </row>
-    <row r="54" spans="1:78" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:78" x14ac:dyDescent="0.3">
       <c r="A54" s="12"/>
       <c r="B54" s="12"/>
       <c r="C54" s="12"/>
@@ -7739,91 +7867,91 @@
       <c r="BY54" s="12"/>
       <c r="BZ54" s="12"/>
     </row>
-    <row r="55" ht="14.4" customHeight="1" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:78" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F55" s="12"/>
     </row>
-    <row r="56" ht="14.4" customHeight="1" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:78" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F56" s="12"/>
     </row>
-    <row r="57" ht="14.4" customHeight="1" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:78" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F57" s="12"/>
     </row>
-    <row r="58" ht="14.4" customHeight="1" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:78" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F58" s="12"/>
     </row>
-    <row r="59" ht="14.4" customHeight="1" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:78" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F59" s="12"/>
     </row>
-    <row r="60" ht="14.4" customHeight="1" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:78" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F60" s="12"/>
     </row>
-    <row r="61" ht="14.4" customHeight="1" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:78" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F61" s="12"/>
     </row>
-    <row r="62" ht="14.4" customHeight="1" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:78" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F62" s="12"/>
     </row>
-    <row r="63" ht="14.4" customHeight="1" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:78" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F63" s="12"/>
     </row>
-    <row r="64" ht="14.4" customHeight="1" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:78" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F64" s="12"/>
     </row>
-    <row r="65" ht="14.4" customHeight="1" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="65" spans="6:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F65" s="12"/>
     </row>
-    <row r="66" ht="14.4" customHeight="1" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="66" spans="6:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F66" s="12"/>
     </row>
-    <row r="67" ht="14.4" customHeight="1" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="67" spans="6:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F67" s="12"/>
     </row>
-    <row r="68" ht="14.4" customHeight="1" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="68" spans="6:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F68" s="12"/>
     </row>
-    <row r="69" ht="14.4" customHeight="1" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="69" spans="6:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F69" s="12"/>
     </row>
-    <row r="70" ht="14.4" customHeight="1" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="70" spans="6:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F70" s="12"/>
     </row>
-    <row r="71" ht="14.4" customHeight="1" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="71" spans="6:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F71" s="12"/>
     </row>
-    <row r="72" ht="14.4" customHeight="1" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="72" spans="6:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F72" s="12"/>
     </row>
-    <row r="73" ht="14.4" customHeight="1" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="73" spans="6:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F73" s="12"/>
     </row>
-    <row r="74" ht="14.4" customHeight="1" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="74" spans="6:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F74" s="12"/>
     </row>
-    <row r="75" ht="14.4" customHeight="1" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="75" spans="6:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F75" s="12"/>
     </row>
-    <row r="76" ht="14.4" customHeight="1" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="76" spans="6:6" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="F76" s="12"/>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="S2" r:id="rId1"/>
-    <hyperlink ref="S3" r:id="rId2"/>
-    <hyperlink ref="S4" r:id="rId3"/>
-    <hyperlink ref="S5" r:id="rId4"/>
-    <hyperlink ref="S6" r:id="rId5"/>
-    <hyperlink ref="S7" r:id="rId6"/>
-    <hyperlink ref="S8" r:id="rId7"/>
-    <hyperlink ref="S9" r:id="rId8"/>
-    <hyperlink ref="S10" r:id="rId9"/>
-    <hyperlink ref="S11" r:id="rId10"/>
-    <hyperlink ref="S12" r:id="rId11"/>
-    <hyperlink ref="S13" r:id="rId12"/>
-    <hyperlink ref="S14" r:id="rId13"/>
-    <hyperlink ref="S15" r:id="rId14"/>
-    <hyperlink ref="S16" r:id="rId15"/>
+    <hyperlink ref="S2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="S3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="S4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="S5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="S6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="S7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="S8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="S9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="S10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="S11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="S12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="S13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="S14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="S15" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="S16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+  <pageSetup orientation="portrait" useFirstPageNumber="1" horizontalDpi="4294967295" verticalDpi="4294967295"/>
 </worksheet>
 </file>
</xml_diff>